<commit_message>
formulas-queries-charts SESSION-02: checkpoint 2 — pivot tables
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbooks/ooxml/pivot-table.xlsx
+++ b/tests/fixtures/workbooks/ooxml/pivot-table.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
   <si>
     <t>Crew</t>
   </si>
@@ -31,6 +31,9 @@
   </si>
   <si>
     <t>Sum of Hours</t>
+  </si>
+  <si>
+    <t>Count of Crew</t>
   </si>
 </sst>
 </file>
@@ -69,12 +72,38 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" recordCount="0"/>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" recordCount="0">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:B4" sheet="Data"/>
+  </cacheSource>
+  <cacheFields count="2">
+    <cacheField name="Crew" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Hours" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="HoursPivot" cacheId="1" dataCaption="Values">
-  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:C5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField axis="axisRow" dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <dataFields count="2">
+    <dataField name="Sum of Hours" fld="1" baseField="0" baseItem="0"/>
+    <dataField name="Count of Crew" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
 </pivotTableDefinition>
 </file>
 
@@ -121,7 +150,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -133,6 +162,9 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -140,6 +172,9 @@
       </c>
       <c r="B4">
         <v>12</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -149,6 +184,9 @@
       <c r="B5">
         <v>6</v>
       </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>